<commit_message>
feat(v3): TTC pasa a columna con nombre propio prob_modelo_cal_smacro (no extra_01)
s3_v3: prob_modelo_cal_smacro (PD calibrada sin macro, lambda=0) como columna
propia junto a prob_modelo_cal/puntuacion_cal; extra_01 vuelve a placeholder.
inference.py (postprocessing+output_fn), testing_out.sql, calibracion_ree.json,
notebook, Diccionario (score, resaltado amarillo) y runbook alineados.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entregables/Artefactos_MLOps_CPPIBKREN_CALIBRADO/Artefactos_mlops_CPPIBKREN/Diccionario_de_Datos_cppibkren.xlsx
+++ b/entregables/Artefactos_MLOps_CPPIBKREN_CALIBRADO/Artefactos_mlops_CPPIBKREN/Diccionario_de_Datos_cppibkren.xlsx
@@ -803,7 +803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I71"/>
+  <dimension ref="B2:I71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="14.5"/>
   <cols>
     <col width="2.6328125" customWidth="1" style="2" min="1" max="1"/>
@@ -995,7 +995,6 @@
       <c r="H12" s="36" t="n"/>
       <c r="I12" s="1" t="n"/>
     </row>
-    <row r="13"/>
     <row r="14" ht="34" customHeight="1">
       <c r="B14" s="7" t="inlineStr">
         <is>
@@ -2498,7 +2497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H84"/>
+  <dimension ref="A2:H85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="14.5"/>
   <cols>
     <col width="2.6328125" customWidth="1" style="2" min="1" max="1"/>
@@ -2680,7 +2679,6 @@
       <c r="G12" s="35" t="n"/>
       <c r="H12" s="36" t="n"/>
     </row>
-    <row r="13"/>
     <row r="14" ht="34" customHeight="1">
       <c r="B14" s="7" t="inlineStr">
         <is>
@@ -3044,32 +3042,28 @@
       <c r="B29" s="43" t="n"/>
       <c r="C29" s="38" t="inlineStr">
         <is>
-          <t>extra_01</t>
+          <t>prob_modelo_cal_smacro</t>
         </is>
       </c>
       <c r="D29" s="38" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>decimal (18,7)</t>
         </is>
       </c>
       <c r="E29" s="39" t="n"/>
       <c r="F29" s="38" t="inlineStr">
         <is>
-          <t>prob_modelo_cal_ttc: PD calibrada TTC (lambda=0)</t>
-        </is>
-      </c>
-      <c r="G29" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">             </t>
-        </is>
-      </c>
+          <t>PD calibrada sin macro (lambda=0)</t>
+        </is>
+      </c>
+      <c r="G29" s="42" t="n"/>
       <c r="H29" s="42" t="n"/>
     </row>
     <row r="30" ht="14.4" customHeight="1">
       <c r="B30" s="8" t="n"/>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>extra_02</t>
+          <t>extra_01</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
@@ -3080,21 +3074,17 @@
       <c r="E30" s="12" t="n"/>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>Variable extra 2</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">             </t>
-        </is>
-      </c>
+          <t>Variable extra 1</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="n"/>
       <c r="H30" s="3" t="n"/>
     </row>
     <row r="31" ht="14.4" customHeight="1">
       <c r="B31" s="8" t="n"/>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>extra_03</t>
+          <t>extra_02</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
@@ -3105,7 +3095,7 @@
       <c r="E31" s="12" t="n"/>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>Variable extra 3</t>
+          <t>Variable extra 2</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -3119,7 +3109,7 @@
       <c r="B32" s="8" t="n"/>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>extra_04</t>
+          <t>extra_03</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
@@ -3130,7 +3120,7 @@
       <c r="E32" s="12" t="n"/>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t>Variable extra 4</t>
+          <t>Variable extra 3</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -3144,7 +3134,7 @@
       <c r="B33" s="8" t="n"/>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>extra_05</t>
+          <t>extra_04</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
@@ -3155,86 +3145,86 @@
       <c r="E33" s="12" t="n"/>
       <c r="F33" s="10" t="inlineStr">
         <is>
+          <t>Variable extra 4</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             </t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="n"/>
+    </row>
+    <row r="34" ht="14.4" customHeight="1">
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>extra_05</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="n"/>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
           <t>Variable extra 5</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">             </t>
         </is>
       </c>
-      <c r="H33" s="3" t="n"/>
-    </row>
-    <row r="34" ht="14.4" customHeight="1">
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>SENTINEL</t>
-        </is>
-      </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>woe_avg_dda_tlc_12m</t>
-        </is>
-      </c>
-      <c r="D34" s="10" t="inlineStr">
-        <is>
-          <t>decimal(18,3)</t>
-        </is>
-      </c>
-      <c r="E34" s="12" t="n"/>
-      <c r="F34" s="14" t="inlineStr">
-        <is>
-          <t>Promedio de días de atraso en servicios de telecomunicaciones U12M</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="n"/>
       <c r="H34" s="3" t="n"/>
     </row>
     <row r="35" ht="14.4" customHeight="1">
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>RENIEC, SUNAT, SUNARP</t>
+          <t>SENTINEL</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>woe_rat_miemsup2r</t>
+          <t>woe_avg_dda_tlc_12m</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>decimal(21,3)</t>
+          <t>decimal(18,3)</t>
         </is>
       </c>
       <c r="E35" s="12" t="n"/>
       <c r="F35" s="14" t="inlineStr">
         <is>
-          <t>Proporción De Miembros Del Hogar Mayores De 18 Años Que Han Completado Estudios Superiores Universitarios</t>
+          <t>Promedio de días de atraso en servicios de telecomunicaciones U12M</t>
         </is>
       </c>
       <c r="G35" s="3" t="n"/>
       <c r="H35" s="3" t="n"/>
     </row>
     <row r="36" ht="14.4" customHeight="1">
-      <c r="B36" s="21" t="inlineStr">
-        <is>
-          <t>GESTIONES</t>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>RENIEC, SUNAT, SUNARP</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>woe_cnt_gestiones_6m</t>
+          <t>woe_rat_miemsup2r</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(21,3)</t>
         </is>
       </c>
       <c r="E36" s="12" t="n"/>
       <c r="F36" s="14" t="inlineStr">
         <is>
-          <t>Cantidad de gestiones de cobranza en los U6M</t>
+          <t>Proporción De Miembros Del Hogar Mayores De 18 Años Que Han Completado Estudios Superiores Universitarios</t>
         </is>
       </c>
       <c r="G36" s="3" t="n"/>
@@ -3243,48 +3233,48 @@
     <row r="37" ht="14.4" customHeight="1">
       <c r="B37" s="21" t="inlineStr">
         <is>
-          <t>RCC</t>
+          <t>GESTIONES</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>woe_std_datraso_rd_u1a</t>
+          <t>woe_cnt_gestiones_6m</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>decimal(23,10)</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E37" s="12" t="n"/>
       <c r="F37" s="14" t="inlineStr">
         <is>
-          <t>Desviación estándar de días de atraso U1A</t>
+          <t>Cantidad de gestiones de cobranza en los U6M</t>
         </is>
       </c>
       <c r="G37" s="3" t="n"/>
       <c r="H37" s="3" t="n"/>
     </row>
     <row r="38" ht="14.4" customHeight="1">
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>IBK</t>
+      <c r="B38" s="21" t="inlineStr">
+        <is>
+          <t>RCC</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>woe_num_inc_sld_tip_pas_12m</t>
+          <t>woe_std_datraso_rd_u1a</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(23,10)</t>
         </is>
       </c>
       <c r="E38" s="12" t="n"/>
       <c r="F38" s="14" t="inlineStr">
         <is>
-          <t>Número de incrementos del saldo en productos pasivos U12M.</t>
+          <t>Desviación estándar de días de atraso U1A</t>
         </is>
       </c>
       <c r="G38" s="3" t="n"/>
@@ -3293,48 +3283,48 @@
     <row r="39" ht="14.4" customHeight="1">
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>RCC</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>woe_max_clfibk_06m</t>
+          <t>woe_num_inc_sld_tip_pas_12m</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,3)</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E39" s="12" t="n"/>
       <c r="F39" s="14" t="inlineStr">
         <is>
-          <t>Máxima clasificación de riesgo en IBK U6M</t>
+          <t>Número de incrementos del saldo en productos pasivos U12M.</t>
         </is>
       </c>
       <c r="G39" s="3" t="n"/>
       <c r="H39" s="3" t="n"/>
     </row>
     <row r="40" ht="14.4" customHeight="1">
-      <c r="B40" s="21" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t>RCC</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>woe_rat_sld_pp_u1m_tc_ibk</t>
+          <t>woe_max_clfibk_06m</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,4)</t>
+          <t>decimal(18,3)</t>
         </is>
       </c>
       <c r="E40" s="12" t="n"/>
       <c r="F40" s="14" t="inlineStr">
         <is>
-          <t>Ratio de saldo en productos PP en 1 mes respecto a TC IBK</t>
+          <t>Máxima clasificación de riesgo en IBK U6M</t>
         </is>
       </c>
       <c r="G40" s="3" t="n"/>
@@ -3343,23 +3333,23 @@
     <row r="41" ht="14.4" customHeight="1">
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>DEPENDIENTE</t>
+          <t>RCC</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>woe_flg_labdp</t>
+          <t>woe_rat_sld_pp_u1m_tc_ibk</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(18,4)</t>
         </is>
       </c>
       <c r="E41" s="12" t="n"/>
       <c r="F41" s="14" t="inlineStr">
         <is>
-          <t>Indicador si el cliente es laboralmente dependiente</t>
+          <t>Ratio de saldo en productos PP en 1 mes respecto a TC IBK</t>
         </is>
       </c>
       <c r="G41" s="3" t="n"/>
@@ -3368,23 +3358,23 @@
     <row r="42" ht="14.4" customHeight="1">
       <c r="B42" s="21" t="inlineStr">
         <is>
-          <t>RCC</t>
+          <t>DEPENDIENTE</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>woe_avg_decrsld12m</t>
+          <t>woe_flg_labdp</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,6)</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E42" s="12" t="n"/>
       <c r="F42" s="14" t="inlineStr">
         <is>
-          <t>Promedio de decremento de saldo U12M</t>
+          <t>Indicador si el cliente es laboralmente dependiente</t>
         </is>
       </c>
       <c r="G42" s="3" t="n"/>
@@ -3398,18 +3388,18 @@
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>woe_cnt_deccorreg_12m</t>
+          <t>woe_avg_decrsld12m</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(18,6)</t>
         </is>
       </c>
       <c r="E43" s="12" t="n"/>
       <c r="F43" s="14" t="inlineStr">
         <is>
-          <t>Cantidad de decrementos corregidos U12M</t>
+          <t>Promedio de decremento de saldo U12M</t>
         </is>
       </c>
       <c r="G43" s="3" t="n"/>
@@ -3423,7 +3413,7 @@
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>woe_max_dias_atraso_no_ibk_3m</t>
+          <t>woe_cnt_deccorreg_12m</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
@@ -3434,7 +3424,7 @@
       <c r="E44" s="12" t="n"/>
       <c r="F44" s="14" t="inlineStr">
         <is>
-          <t>Máximo días de atraso en entidades no IBK U3M</t>
+          <t>Cantidad de decrementos corregidos U12M</t>
         </is>
       </c>
       <c r="G44" s="3" t="n"/>
@@ -3443,23 +3433,23 @@
     <row r="45" ht="14.4" customHeight="1">
       <c r="B45" s="21" t="inlineStr">
         <is>
-          <t>IBK</t>
+          <t>RCC</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>woe_avg_diamorasldppibk_12m</t>
+          <t>woe_max_dias_atraso_no_ibk_3m</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,3)</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E45" s="12" t="n"/>
       <c r="F45" s="14" t="inlineStr">
         <is>
-          <t>Promedio de días de mora en saldo PP IBK U12M</t>
+          <t>Máximo días de atraso en entidades no IBK U3M</t>
         </is>
       </c>
       <c r="G45" s="3" t="n"/>
@@ -3468,23 +3458,23 @@
     <row r="46" ht="14.4" customHeight="1">
       <c r="B46" s="21" t="inlineStr">
         <is>
-          <t>SENTINEL</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>woe_mto_dda_otr_emp_12m</t>
+          <t>woe_avg_diamorasldppibk_12m</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,6)</t>
+          <t>decimal(18,3)</t>
         </is>
       </c>
       <c r="E46" s="12" t="n"/>
       <c r="F46" s="14" t="inlineStr">
         <is>
-          <t>Monto de deuda con otros empleadores U12M</t>
+          <t>Promedio de días de mora en saldo PP IBK U12M</t>
         </is>
       </c>
       <c r="G46" s="3" t="n"/>
@@ -3493,23 +3483,23 @@
     <row r="47" ht="14.4" customHeight="1">
       <c r="B47" s="21" t="inlineStr">
         <is>
-          <t>RCC</t>
+          <t>SENTINEL</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>woe_ant_profesional</t>
+          <t>woe_mto_dda_otr_emp_12m</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(18,6)</t>
         </is>
       </c>
       <c r="E47" s="12" t="n"/>
       <c r="F47" s="14" t="inlineStr">
         <is>
-          <t>Antigüedad profesional en años</t>
+          <t>Monto de deuda con otros empleadores U12M</t>
         </is>
       </c>
       <c r="G47" s="3" t="n"/>
@@ -3523,18 +3513,18 @@
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>woe_mto_totalrec06m</t>
+          <t>woe_ant_profesional</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,3)</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E48" s="12" t="n"/>
       <c r="F48" s="14" t="inlineStr">
         <is>
-          <t>Monto total recibido U6M</t>
+          <t>Antigüedad profesional en años</t>
         </is>
       </c>
       <c r="G48" s="3" t="n"/>
@@ -3543,12 +3533,12 @@
     <row r="49" ht="14.4" customHeight="1">
       <c r="B49" s="21" t="inlineStr">
         <is>
-          <t>PASIVOS</t>
+          <t>RCC</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>woe_rat_maxsldppibk_03m</t>
+          <t>woe_mto_totalrec06m</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
@@ -3559,7 +3549,7 @@
       <c r="E49" s="12" t="n"/>
       <c r="F49" s="14" t="inlineStr">
         <is>
-          <t>Ratio máximo de saldo PP IBK U3M</t>
+          <t>Monto total recibido U6M</t>
         </is>
       </c>
       <c r="G49" s="3" t="n"/>
@@ -3568,48 +3558,48 @@
     <row r="50" ht="14.4" customHeight="1">
       <c r="B50" s="21" t="inlineStr">
         <is>
-          <t>RCC</t>
+          <t>PASIVOS</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>woe_rat_comparacion_u1m_u12m</t>
+          <t>woe_rat_maxsldppibk_03m</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,4)</t>
+          <t>decimal(18,3)</t>
         </is>
       </c>
       <c r="E50" s="12" t="n"/>
       <c r="F50" s="14" t="inlineStr">
         <is>
-          <t>Ratio entre el saldo del último mes y el promedio U12M.</t>
+          <t>Ratio máximo de saldo PP IBK U3M</t>
         </is>
       </c>
       <c r="G50" s="3" t="n"/>
       <c r="H50" s="3" t="n"/>
     </row>
     <row r="51" ht="14.4" customHeight="1">
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>IBK</t>
+      <c r="B51" s="21" t="inlineStr">
+        <is>
+          <t>RCC</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>woe_ant_primer_producto</t>
+          <t>woe_rat_comparacion_u1m_u12m</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(18,4)</t>
         </is>
       </c>
       <c r="E51" s="12" t="n"/>
       <c r="F51" s="14" t="inlineStr">
         <is>
-          <t>Antigüedad del primer producto financiero en meses</t>
+          <t>Ratio entre el saldo del último mes y el promedio U12M.</t>
         </is>
       </c>
       <c r="G51" s="3" t="n"/>
@@ -3618,52 +3608,52 @@
     <row r="52" ht="14.4" customHeight="1">
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>PASIVOS</t>
+          <t>IBK</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>woe_min_pasctasld_12m</t>
+          <t>woe_ant_primer_producto</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,3)</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E52" s="12" t="n"/>
       <c r="F52" s="14" t="inlineStr">
         <is>
-          <t>Saldo mínimo en cuenta sueldo U12M</t>
-        </is>
-      </c>
-      <c r="G52" s="9" t="n"/>
-      <c r="H52" s="9" t="n"/>
+          <t>Antigüedad del primer producto financiero en meses</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="n"/>
+      <c r="H52" s="3" t="n"/>
     </row>
     <row r="53" ht="14.4" customHeight="1">
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>RCC</t>
+          <t>PASIVOS</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>woe_avg_slddispefpn_u6m</t>
+          <t>woe_min_pasctasld_12m</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>decimal(23,10)</t>
+          <t>decimal(18,3)</t>
         </is>
       </c>
       <c r="E53" s="12" t="n"/>
       <c r="F53" s="14" t="inlineStr">
         <is>
-          <t>Promedio de saldo disponible efectivo U6M</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="n"/>
-      <c r="H53" s="3" t="n"/>
+          <t>Saldo mínimo en cuenta sueldo U12M</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="n"/>
+      <c r="H53" s="9" t="n"/>
     </row>
     <row r="54" ht="14.4" customHeight="1">
       <c r="B54" s="8" t="inlineStr">
@@ -3673,18 +3663,18 @@
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>woe_sld_beta_pc_pp_1a</t>
+          <t>woe_avg_slddispefpn_u6m</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,6)</t>
+          <t>decimal(23,10)</t>
         </is>
       </c>
       <c r="E54" s="12" t="n"/>
       <c r="F54" s="14" t="inlineStr">
         <is>
-          <t>Sensibilidad/variabilidad del saldo personal U1A.</t>
+          <t>Promedio de saldo disponible efectivo U6M</t>
         </is>
       </c>
       <c r="G54" s="3" t="n"/>
@@ -3693,23 +3683,23 @@
     <row r="55" ht="14.4" customHeight="1">
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>SUNARP</t>
+          <t>RCC</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>woe_num_vehiculos</t>
+          <t>woe_sld_beta_pc_pp_1a</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(18,6)</t>
         </is>
       </c>
       <c r="E55" s="12" t="n"/>
       <c r="F55" s="14" t="inlineStr">
         <is>
-          <t>Número de vehículos registrados</t>
+          <t>Sensibilidad/variabilidad del saldo personal U1A.</t>
         </is>
       </c>
       <c r="G55" s="3" t="n"/>
@@ -3718,12 +3708,12 @@
     <row r="56" ht="14.4" customHeight="1">
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>RENIEC</t>
+          <t>SUNARP</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>woe_num_edad</t>
+          <t>woe_num_vehiculos</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
@@ -3734,7 +3724,7 @@
       <c r="E56" s="12" t="n"/>
       <c r="F56" s="14" t="inlineStr">
         <is>
-          <t>Edad del cliente</t>
+          <t>Número de vehículos registrados</t>
         </is>
       </c>
       <c r="G56" s="3" t="n"/>
@@ -3743,23 +3733,23 @@
     <row r="57" ht="14.4" customHeight="1">
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>RCC</t>
+          <t>RENIEC</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>woe_var_ent_dist_rd_1a</t>
+          <t>woe_num_edad</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,6)</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E57" s="12" t="n"/>
       <c r="F57" s="14" t="inlineStr">
         <is>
-          <t>Variabilidad en la cantidad de entidades financieras con productos revolventes en el último año. Mide dispersión de relaciones crediticias.</t>
+          <t>Edad del cliente</t>
         </is>
       </c>
       <c r="G57" s="3" t="n"/>
@@ -3773,18 +3763,18 @@
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>woe_max_dda_pp_rat_9m</t>
+          <t>woe_var_ent_dist_rd_1a</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>decimal(23,10)</t>
+          <t>decimal(18,6)</t>
         </is>
       </c>
       <c r="E58" s="12" t="n"/>
       <c r="F58" s="14" t="inlineStr">
         <is>
-          <t>Máxima variación de deuda PP U9M</t>
+          <t>Variabilidad en la cantidad de entidades financieras con productos revolventes en el último año. Mide dispersión de relaciones crediticias.</t>
         </is>
       </c>
       <c r="G58" s="3" t="n"/>
@@ -3793,23 +3783,23 @@
     <row r="59" ht="14.4" customHeight="1">
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>PASIVOS</t>
+          <t>RCC</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>woe_rat_actpas_03m</t>
+          <t>woe_max_dda_pp_rat_9m</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,6)</t>
+          <t>decimal(23,10)</t>
         </is>
       </c>
       <c r="E59" s="12" t="n"/>
       <c r="F59" s="14" t="inlineStr">
         <is>
-          <t>Ratio activos/pasivos U3M</t>
+          <t>Máxima variación de deuda PP U9M</t>
         </is>
       </c>
       <c r="G59" s="3" t="n"/>
@@ -3818,73 +3808,73 @@
     <row r="60" ht="14.4" customHeight="1">
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>RCC</t>
+          <t>PASIVOS</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>woe_avg_rat_dispefpnj_u1a</t>
+          <t>woe_rat_actpas_03m</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,3)</t>
+          <t>decimal(18,6)</t>
         </is>
       </c>
       <c r="E60" s="12" t="n"/>
       <c r="F60" s="14" t="inlineStr">
         <is>
-          <t>Promedio del ratio de saldo disponible efectivo U1A</t>
+          <t>Ratio activos/pasivos U3M</t>
         </is>
       </c>
       <c r="G60" s="3" t="n"/>
       <c r="H60" s="3" t="n"/>
     </row>
     <row r="61" ht="14.4" customHeight="1">
-      <c r="B61" s="21" t="inlineStr">
+      <c r="B61" s="8" t="inlineStr">
         <is>
           <t>RCC</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>woe_num_titulo_prof</t>
+          <t>woe_avg_rat_dispefpnj_u1a</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(18,3)</t>
         </is>
       </c>
       <c r="E61" s="12" t="n"/>
       <c r="F61" s="14" t="inlineStr">
         <is>
-          <t>Número de títulos profesionales del cliente.</t>
+          <t>Promedio del ratio de saldo disponible efectivo U1A</t>
         </is>
       </c>
       <c r="G61" s="3" t="n"/>
       <c r="H61" s="3" t="n"/>
     </row>
     <row r="62" ht="14.4" customHeight="1">
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B62" s="21" t="inlineStr">
         <is>
           <t>RCC</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>woe_rat_saldo_rt_t1_t12</t>
+          <t>woe_num_titulo_prof</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>decimal(21,3)</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E62" s="12" t="n"/>
       <c r="F62" s="14" t="inlineStr">
         <is>
-          <t>Ratio entre saldo reciente y saldo máximo anual en productos rotativos</t>
+          <t>Número de títulos profesionales del cliente.</t>
         </is>
       </c>
       <c r="G62" s="3" t="n"/>
@@ -3898,57 +3888,57 @@
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>woe_porc_max_sldrsg_06m</t>
+          <t>woe_rat_saldo_rt_t1_t12</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,3)</t>
+          <t>decimal(21,3)</t>
         </is>
       </c>
       <c r="E63" s="12" t="n"/>
       <c r="F63" s="14" t="inlineStr">
         <is>
-          <t>Porcentaje máximo de saldo en productos RD U6M</t>
+          <t>Ratio entre saldo reciente y saldo máximo anual en productos rotativos</t>
         </is>
       </c>
       <c r="G63" s="3" t="n"/>
       <c r="H63" s="3" t="n"/>
     </row>
     <row r="64" ht="14.4" customHeight="1">
-      <c r="B64" s="21" t="inlineStr">
+      <c r="B64" s="8" t="inlineStr">
         <is>
           <t>RCC</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>woe_cnt_dectctotal_12m</t>
+          <t>woe_porc_max_sldrsg_06m</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(18,3)</t>
         </is>
       </c>
       <c r="E64" s="12" t="n"/>
       <c r="F64" s="14" t="inlineStr">
         <is>
-          <t>Cantidad de decrementos totales en tarjeta de crédito U12M</t>
+          <t>Porcentaje máximo de saldo en productos RD U6M</t>
         </is>
       </c>
       <c r="G64" s="3" t="n"/>
       <c r="H64" s="3" t="n"/>
     </row>
     <row r="65" ht="14.4" customHeight="1">
-      <c r="B65" s="8" t="inlineStr">
-        <is>
-          <t>PASIVOS</t>
+      <c r="B65" s="21" t="inlineStr">
+        <is>
+          <t>RCC</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>woe_flg_pasibk</t>
+          <t>woe_cnt_dectctotal_12m</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
@@ -3959,7 +3949,7 @@
       <c r="E65" s="12" t="n"/>
       <c r="F65" s="14" t="inlineStr">
         <is>
-          <t>Indicador si el cliente tiene pasivos en IBK</t>
+          <t>Cantidad de decrementos totales en tarjeta de crédito U12M</t>
         </is>
       </c>
       <c r="G65" s="3" t="n"/>
@@ -3968,73 +3958,73 @@
     <row r="66" ht="14.4" customHeight="1">
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>RCC</t>
+          <t>PASIVOS</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>woe_porc_avg_sld_rd_6m</t>
+          <t>woe_flg_pasibk</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>decimal(23,10)</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E66" s="12" t="n"/>
       <c r="F66" s="14" t="inlineStr">
         <is>
-          <t>Porcentaje promedio de saldo en productos RD U6M</t>
+          <t>Indicador si el cliente tiene pasivos en IBK</t>
         </is>
       </c>
       <c r="G66" s="3" t="n"/>
       <c r="H66" s="3" t="n"/>
     </row>
     <row r="67" ht="14.4" customHeight="1">
-      <c r="B67" s="21" t="inlineStr">
+      <c r="B67" s="8" t="inlineStr">
         <is>
           <t>RCC</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>woe_med_sld_sa_hip_3i_6m</t>
+          <t>woe_porc_avg_sld_rd_6m</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,3)</t>
+          <t>decimal(23,10)</t>
         </is>
       </c>
       <c r="E67" s="12" t="n"/>
       <c r="F67" s="14" t="inlineStr">
         <is>
-          <t>Mediana del saldo en productos hipotecarios U6M</t>
+          <t>Porcentaje promedio de saldo en productos RD U6M</t>
         </is>
       </c>
       <c r="G67" s="3" t="n"/>
       <c r="H67" s="3" t="n"/>
     </row>
     <row r="68" ht="14.4" customHeight="1">
-      <c r="B68" s="8" t="inlineStr">
-        <is>
-          <t>SALDOS</t>
+      <c r="B68" s="21" t="inlineStr">
+        <is>
+          <t>RCC</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>woe_cnt_atraso_01_aj</t>
+          <t>woe_med_sld_sa_hip_3i_6m</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(18,3)</t>
         </is>
       </c>
       <c r="E68" s="12" t="n"/>
       <c r="F68" s="14" t="inlineStr">
         <is>
-          <t>Máximo de días de atraso en el mes 1, para clientes sin atraso en el mes evaluado (mes 0).</t>
+          <t>Mediana del saldo en productos hipotecarios U6M</t>
         </is>
       </c>
       <c r="G68" s="3" t="n"/>
@@ -4043,12 +4033,12 @@
     <row r="69" ht="14.4" customHeight="1">
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>RCC</t>
+          <t>SALDOS</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>woe_num_inmuebles</t>
+          <t>woe_cnt_atraso_01_aj</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
@@ -4059,7 +4049,7 @@
       <c r="E69" s="12" t="n"/>
       <c r="F69" s="14" t="inlineStr">
         <is>
-          <t>Número de propiedades inscritas en SUNARP</t>
+          <t>Máximo de días de atraso en el mes 1, para clientes sin atraso en el mes evaluado (mes 0).</t>
         </is>
       </c>
       <c r="G69" s="3" t="n"/>
@@ -4073,18 +4063,18 @@
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>woe_avg_trxtot12m</t>
+          <t>woe_num_inmuebles</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,3)</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E70" s="12" t="n"/>
       <c r="F70" s="14" t="inlineStr">
         <is>
-          <t>Promedio de transacciones totales U12M</t>
+          <t>Número de propiedades inscritas en SUNARP</t>
         </is>
       </c>
       <c r="G70" s="3" t="n"/>
@@ -4098,18 +4088,18 @@
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>woe_porc_avg_pctusotctot_u1a</t>
+          <t>woe_avg_trxtot12m</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>decimal(23,10)</t>
+          <t>decimal(18,3)</t>
         </is>
       </c>
       <c r="E71" s="12" t="n"/>
       <c r="F71" s="14" t="inlineStr">
         <is>
-          <t>Porcentaje promedio de uso de TC U1A</t>
+          <t>Promedio de transacciones totales U12M</t>
         </is>
       </c>
       <c r="G71" s="3" t="n"/>
@@ -4118,23 +4108,23 @@
     <row r="72" ht="14.4" customHeight="1">
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>HPC</t>
+          <t>RCC</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>woe_cnt_dias_adelanto_atraso</t>
+          <t>woe_porc_avg_pctusotctot_u1a</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(23,10)</t>
         </is>
       </c>
       <c r="E72" s="12" t="n"/>
       <c r="F72" s="14" t="inlineStr">
         <is>
-          <t>Dias entre pago y vencimiento (negativo=anticipado, positivo=atrasado).</t>
+          <t>Porcentaje promedio de uso de TC U1A</t>
         </is>
       </c>
       <c r="G72" s="3" t="n"/>
@@ -4143,98 +4133,98 @@
     <row r="73" ht="14.4" customHeight="1">
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>RCC</t>
+          <t>HPC</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>woe_cnt_mespeornorssff_12m</t>
+          <t>woe_cnt_dias_adelanto_atraso</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,3)</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E73" s="12" t="n"/>
       <c r="F73" s="14" t="inlineStr">
         <is>
-          <t>Cantidad de meses desde peor clasificación normal en SSFF</t>
+          <t>Dias entre pago y vencimiento (negativo=anticipado, positivo=atrasado).</t>
         </is>
       </c>
       <c r="G73" s="3" t="n"/>
       <c r="H73" s="3" t="n"/>
     </row>
     <row r="74" ht="14.4" customHeight="1">
-      <c r="B74" s="21" t="inlineStr">
+      <c r="B74" s="8" t="inlineStr">
         <is>
           <t>RCC</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>woe_rat_svotrppeallsf_3m</t>
+          <t>woe_cnt_mespeornorssff_12m</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>decimal(23,10)</t>
+          <t>decimal(18,3)</t>
         </is>
       </c>
       <c r="E74" s="12" t="n"/>
       <c r="F74" s="14" t="inlineStr">
         <is>
-          <t>Ratio de saldo vigente en otras entidades U3M</t>
+          <t>Cantidad de meses desde peor clasificación normal en SSFF</t>
         </is>
       </c>
       <c r="G74" s="3" t="n"/>
       <c r="H74" s="3" t="n"/>
     </row>
     <row r="75" ht="14.4" customHeight="1">
-      <c r="B75" s="8" t="inlineStr">
+      <c r="B75" s="21" t="inlineStr">
         <is>
           <t>RCC</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
         <is>
-          <t>woe_med_dec_sld_tarj_3i_6m</t>
+          <t>woe_rat_svotrppeallsf_3m</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>decimal(18,3)</t>
+          <t>decimal(23,10)</t>
         </is>
       </c>
       <c r="E75" s="12" t="n"/>
       <c r="F75" s="14" t="inlineStr">
         <is>
-          <t>Mediana del decrecimiento del saldo en tarjetas de crédito en 3 instancias U6M.</t>
+          <t>Ratio de saldo vigente en otras entidades U3M</t>
         </is>
       </c>
       <c r="G75" s="3" t="n"/>
       <c r="H75" s="3" t="n"/>
     </row>
     <row r="76" ht="14.4" customHeight="1">
-      <c r="B76" s="21" t="inlineStr">
-        <is>
-          <t>INTERCORP</t>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>RCC</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>woe_trf_mtomax_grifos_pos12m</t>
+          <t>woe_med_dec_sld_tarj_3i_6m</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>decimal(18,3)</t>
         </is>
       </c>
       <c r="E76" s="12" t="n"/>
       <c r="F76" s="14" t="inlineStr">
         <is>
-          <t>Monto máximo de transacción POS en rubro Grifos U12M</t>
+          <t>Mediana del decrecimiento del saldo en tarjetas de crédito en 3 instancias U6M.</t>
         </is>
       </c>
       <c r="G76" s="3" t="n"/>
@@ -4248,7 +4238,7 @@
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>woe_trf_far_mtomax_med_12m</t>
+          <t>woe_trf_mtomax_grifos_pos12m</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
@@ -4259,7 +4249,7 @@
       <c r="E77" s="12" t="n"/>
       <c r="F77" s="14" t="inlineStr">
         <is>
-          <t>Monto neto máximo de compra en Farmacias Peruanas - Medicamento U12M</t>
+          <t>Monto máximo de transacción POS en rubro Grifos U12M</t>
         </is>
       </c>
       <c r="G77" s="3" t="n"/>
@@ -4273,7 +4263,7 @@
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>woe_trf_mtot_tc_retail_pos1m</t>
+          <t>woe_trf_far_mtomax_med_12m</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr">
@@ -4284,7 +4274,7 @@
       <c r="E78" s="12" t="n"/>
       <c r="F78" s="14" t="inlineStr">
         <is>
-          <t>Monto total consumido por el cliente con TC en transacciones Retail/POS U1M</t>
+          <t>Monto neto máximo de compra en Farmacias Peruanas - Medicamento U12M</t>
         </is>
       </c>
       <c r="G78" s="3" t="n"/>
@@ -4298,7 +4288,7 @@
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>woe_trf_prm_restaur_pos_6m</t>
+          <t>woe_trf_mtot_tc_retail_pos1m</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
@@ -4309,7 +4299,7 @@
       <c r="E79" s="12" t="n"/>
       <c r="F79" s="14" t="inlineStr">
         <is>
-          <t>Monto promedio por transacción en Restaurantes U6M</t>
+          <t>Monto total consumido por el cliente con TC en transacciones Retail/POS U1M</t>
         </is>
       </c>
       <c r="G79" s="3" t="n"/>
@@ -4323,7 +4313,7 @@
       </c>
       <c r="C80" s="10" t="inlineStr">
         <is>
-          <t>woe_trf_mtoprm_altagama_12m</t>
+          <t>woe_trf_prm_restaur_pos_6m</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
@@ -4334,7 +4324,7 @@
       <c r="E80" s="12" t="n"/>
       <c r="F80" s="14" t="inlineStr">
         <is>
-          <t>Monto promedio de transacciones/productos de alta gama U12M</t>
+          <t>Monto promedio por transacción en Restaurantes U6M</t>
         </is>
       </c>
       <c r="G80" s="3" t="n"/>
@@ -4348,7 +4338,7 @@
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>woe_trf_mto_salud_u24m</t>
+          <t>woe_trf_mtoprm_altagama_12m</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
@@ -4359,36 +4349,36 @@
       <c r="E81" s="12" t="n"/>
       <c r="F81" s="14" t="inlineStr">
         <is>
-          <t>Monto total de consumo del cliente en sector Salud U24M</t>
+          <t>Monto promedio de transacciones/productos de alta gama U12M</t>
         </is>
       </c>
       <c r="G81" s="3" t="n"/>
       <c r="H81" s="3" t="n"/>
     </row>
     <row r="82">
-      <c r="B82" s="43" t="inlineStr">
-        <is>
-          <t>MACRO</t>
-        </is>
-      </c>
-      <c r="C82" s="42" t="inlineStr">
-        <is>
-          <t>trf_macro01</t>
-        </is>
-      </c>
-      <c r="D82" s="44" t="inlineStr">
-        <is>
-          <t>decimal(38,14)</t>
-        </is>
-      </c>
-      <c r="E82" s="42" t="n"/>
-      <c r="F82" s="42" t="inlineStr">
-        <is>
-          <t>Factor sistemico f_t (Vasicek) aplicado en el PIT</t>
-        </is>
-      </c>
-      <c r="G82" s="42" t="n"/>
-      <c r="H82" s="42" t="n"/>
+      <c r="B82" s="21" t="inlineStr">
+        <is>
+          <t>INTERCORP</t>
+        </is>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>woe_trf_mto_salud_u24m</t>
+        </is>
+      </c>
+      <c r="D82" s="10" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E82" s="12" t="n"/>
+      <c r="F82" s="14" t="inlineStr">
+        <is>
+          <t>Monto total de consumo del cliente en sector Salud U24M</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="n"/>
+      <c r="H82" s="3" t="n"/>
     </row>
     <row r="83">
       <c r="B83" s="43" t="inlineStr">
@@ -4398,7 +4388,7 @@
       </c>
       <c r="C83" s="42" t="inlineStr">
         <is>
-          <t>trf_macro02</t>
+          <t>trf_macro01</t>
         </is>
       </c>
       <c r="D83" s="44" t="inlineStr">
@@ -4409,32 +4399,57 @@
       <c r="E83" s="42" t="n"/>
       <c r="F83" s="42" t="inlineStr">
         <is>
-          <t>Macro transformada: media de porc_ipc de T-10 a T-5</t>
+          <t>Factor sistemico f_t (Vasicek) aplicado en el PIT</t>
         </is>
       </c>
       <c r="G83" s="42" t="n"/>
       <c r="H83" s="42" t="n"/>
     </row>
     <row r="84" ht="14.4" customHeight="1">
-      <c r="B84" s="8" t="n"/>
-      <c r="C84" s="10" t="inlineStr">
+      <c r="B84" s="43" t="inlineStr">
+        <is>
+          <t>MACRO</t>
+        </is>
+      </c>
+      <c r="C84" s="42" t="inlineStr">
+        <is>
+          <t>trf_macro02</t>
+        </is>
+      </c>
+      <c r="D84" s="44" t="inlineStr">
+        <is>
+          <t>decimal(38,14)</t>
+        </is>
+      </c>
+      <c r="E84" s="42" t="n"/>
+      <c r="F84" s="42" t="inlineStr">
+        <is>
+          <t>Macro transformada: media de porc_ipc de T-10 a T-5</t>
+        </is>
+      </c>
+      <c r="G84" s="42" t="n"/>
+      <c r="H84" s="42" t="n"/>
+    </row>
+    <row r="85">
+      <c r="B85" s="8" t="n"/>
+      <c r="C85" s="10" t="inlineStr">
         <is>
           <t>p_codmes</t>
         </is>
       </c>
-      <c r="D84" s="10" t="inlineStr">
+      <c r="D85" s="10" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="E84" s="12" t="n"/>
-      <c r="F84" s="14" t="inlineStr">
+      <c r="E85" s="12" t="n"/>
+      <c r="F85" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Partición mensual en yyyymm.  </t>
         </is>
       </c>
-      <c r="G84" s="3" t="n"/>
-      <c r="H84" s="3" t="n"/>
+      <c r="G85" s="3" t="n"/>
+      <c r="H85" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">

</xml_diff>